<commit_message>
update w/ XT60 + silkscreen improvement
</commit_message>
<xml_diff>
--- a/BOM.xlsx
+++ b/BOM.xlsx
@@ -20,7 +20,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="74" uniqueCount="74">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="76" uniqueCount="76">
   <si>
     <t xml:space="preserve">Item</t>
   </si>
@@ -94,12 +94,18 @@
     <t xml:space="preserve">https://www.lcsc.com/product-detail/C2913282.html</t>
   </si>
   <si>
-    <t xml:space="preserve">XT60PW-F (XT60 headers)</t>
+    <t xml:space="preserve">XT60PW-F (XT60 female headers)</t>
   </si>
   <si>
     <t xml:space="preserve">https://www.lcsc.com/product-detail/C428722.html</t>
   </si>
   <si>
+    <t xml:space="preserve">XT60PW-M (XT60 male header)</t>
+  </si>
+  <si>
+    <t xml:space="preserve">https://www.lcsc.com/product-detail/C98732.html</t>
+  </si>
+  <si>
     <t xml:space="preserve">S3B-XH-A(LF)(SN) (XH 3P R/A)</t>
   </si>
   <si>
@@ -214,7 +220,7 @@
     <t xml:space="preserve">https://www.lcsc.com/product-detail/C2998928.html</t>
   </si>
   <si>
-    <t xml:space="preserve">Temperature sensor</t>
+    <t xml:space="preserve">TMP100NA/3K (temp sensor)</t>
   </si>
   <si>
     <t xml:space="preserve">https://www.lcsc.com/product-detail/C31810.html</t>
@@ -475,7 +481,7 @@
   <sheetPr filterMode="false">
     <pageSetUpPr fitToPage="false"/>
   </sheetPr>
-  <dimension ref="A1:F39"/>
+  <dimension ref="A1:F40"/>
   <sheetFormatPr defaultColWidth="11.53515625" defaultRowHeight="12.8" customHeight="false" zeroHeight="false" outlineLevelRow="0" outlineLevelCol="0"/>
   <cols>
     <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="1" min="1" style="1" width="38.67"/>
@@ -668,14 +674,14 @@
         <v>0.5489</v>
       </c>
       <c r="C11" s="1" t="n">
-        <v>2</v>
+        <v>1</v>
       </c>
       <c r="D11" s="1" t="s">
         <v>25</v>
       </c>
       <c r="E11" s="2" t="n">
         <f aca="false">B11*C11</f>
-        <v>1.0978</v>
+        <v>0.5489</v>
       </c>
     </row>
     <row r="12" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -683,7 +689,7 @@
         <v>26</v>
       </c>
       <c r="B12" s="2" t="n">
-        <v>0.0915</v>
+        <v>0.52</v>
       </c>
       <c r="C12" s="1" t="n">
         <v>1</v>
@@ -692,7 +698,8 @@
         <v>27</v>
       </c>
       <c r="E12" s="2" t="n">
-        <v>0.92</v>
+        <f aca="false">B12*C12</f>
+        <v>0.52</v>
       </c>
     </row>
     <row r="13" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -700,16 +707,16 @@
         <v>28</v>
       </c>
       <c r="B13" s="2" t="n">
-        <v>0.153</v>
+        <v>0.0915</v>
       </c>
       <c r="C13" s="1" t="n">
-        <v>2</v>
+        <v>1</v>
       </c>
       <c r="D13" s="1" t="s">
         <v>29</v>
       </c>
       <c r="E13" s="2" t="n">
-        <v>0.77</v>
+        <v>0.92</v>
       </c>
     </row>
     <row r="14" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -717,17 +724,16 @@
         <v>30</v>
       </c>
       <c r="B14" s="2" t="n">
-        <v>0.8048</v>
+        <v>0.153</v>
       </c>
       <c r="C14" s="1" t="n">
-        <v>1</v>
+        <v>2</v>
       </c>
       <c r="D14" s="1" t="s">
         <v>31</v>
       </c>
       <c r="E14" s="2" t="n">
-        <f aca="false">B14*C14</f>
-        <v>0.8048</v>
+        <v>0.77</v>
       </c>
     </row>
     <row r="15" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -735,7 +741,7 @@
         <v>32</v>
       </c>
       <c r="B15" s="2" t="n">
-        <v>0.3364</v>
+        <v>0.8048</v>
       </c>
       <c r="C15" s="1" t="n">
         <v>1</v>
@@ -744,7 +750,8 @@
         <v>33</v>
       </c>
       <c r="E15" s="2" t="n">
-        <v>1.68</v>
+        <f aca="false">B15*C15</f>
+        <v>0.8048</v>
       </c>
     </row>
     <row r="16" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -752,16 +759,16 @@
         <v>34</v>
       </c>
       <c r="B16" s="2" t="n">
-        <v>0.0191</v>
+        <v>0.3364</v>
       </c>
       <c r="C16" s="1" t="n">
-        <v>12</v>
+        <v>1</v>
       </c>
       <c r="D16" s="1" t="s">
         <v>35</v>
       </c>
       <c r="E16" s="2" t="n">
-        <v>0.96</v>
+        <v>1.68</v>
       </c>
     </row>
     <row r="17" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -769,16 +776,16 @@
         <v>36</v>
       </c>
       <c r="B17" s="2" t="n">
-        <v>0.0232</v>
+        <v>0.0191</v>
       </c>
       <c r="C17" s="1" t="n">
-        <v>2</v>
+        <v>12</v>
       </c>
       <c r="D17" s="1" t="s">
         <v>37</v>
       </c>
       <c r="E17" s="2" t="n">
-        <v>0.46</v>
+        <v>0.96</v>
       </c>
     </row>
     <row r="18" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -786,7 +793,7 @@
         <v>38</v>
       </c>
       <c r="B18" s="2" t="n">
-        <v>0.0225</v>
+        <v>0.0232</v>
       </c>
       <c r="C18" s="1" t="n">
         <v>2</v>
@@ -795,7 +802,7 @@
         <v>39</v>
       </c>
       <c r="E18" s="2" t="n">
-        <v>0.45</v>
+        <v>0.46</v>
       </c>
     </row>
     <row r="19" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -803,16 +810,16 @@
         <v>40</v>
       </c>
       <c r="B19" s="2" t="n">
-        <v>0.0083</v>
+        <v>0.0225</v>
       </c>
       <c r="C19" s="1" t="n">
-        <v>14</v>
+        <v>2</v>
       </c>
       <c r="D19" s="1" t="s">
         <v>41</v>
       </c>
       <c r="E19" s="2" t="n">
-        <v>0.42</v>
+        <v>0.45</v>
       </c>
     </row>
     <row r="20" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -820,16 +827,16 @@
         <v>42</v>
       </c>
       <c r="B20" s="2" t="n">
-        <v>0.0538</v>
+        <v>0.0083</v>
       </c>
       <c r="C20" s="1" t="n">
-        <v>1</v>
+        <v>14</v>
       </c>
       <c r="D20" s="1" t="s">
         <v>43</v>
       </c>
       <c r="E20" s="2" t="n">
-        <v>0.54</v>
+        <v>0.42</v>
       </c>
     </row>
     <row r="21" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -837,36 +844,36 @@
         <v>44</v>
       </c>
       <c r="B21" s="2" t="n">
-        <v>0.0334</v>
+        <v>0.0538</v>
       </c>
       <c r="C21" s="1" t="n">
-        <v>4</v>
+        <v>1</v>
       </c>
       <c r="D21" s="1" t="s">
         <v>45</v>
       </c>
       <c r="E21" s="2" t="n">
-        <v>0.67</v>
-      </c>
-      <c r="F21" s="1" t="s">
-        <v>46</v>
+        <v>0.54</v>
       </c>
     </row>
     <row r="22" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A22" s="1" t="s">
+        <v>46</v>
+      </c>
+      <c r="B22" s="2" t="n">
+        <v>0.0334</v>
+      </c>
+      <c r="C22" s="1" t="n">
+        <v>4</v>
+      </c>
+      <c r="D22" s="1" t="s">
         <v>47</v>
       </c>
-      <c r="B22" s="2" t="n">
-        <v>0.0137</v>
-      </c>
-      <c r="C22" s="1" t="n">
-        <v>2</v>
-      </c>
-      <c r="D22" s="1" t="s">
+      <c r="E22" s="2" t="n">
+        <v>0.67</v>
+      </c>
+      <c r="F22" s="1" t="s">
         <v>48</v>
-      </c>
-      <c r="E22" s="2" t="n">
-        <v>0.69</v>
       </c>
     </row>
     <row r="23" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -874,36 +881,36 @@
         <v>49</v>
       </c>
       <c r="B23" s="2" t="n">
-        <v>0.0059</v>
+        <v>0.0137</v>
       </c>
       <c r="C23" s="1" t="n">
-        <v>7</v>
+        <v>2</v>
       </c>
       <c r="D23" s="1" t="s">
         <v>50</v>
       </c>
       <c r="E23" s="2" t="n">
-        <v>0.59</v>
-      </c>
-      <c r="F23" s="4" t="s">
-        <v>51</v>
+        <v>0.69</v>
       </c>
     </row>
     <row r="24" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A24" s="1" t="s">
+        <v>51</v>
+      </c>
+      <c r="B24" s="2" t="n">
+        <v>0.0059</v>
+      </c>
+      <c r="C24" s="1" t="n">
+        <v>7</v>
+      </c>
+      <c r="D24" s="1" t="s">
         <v>52</v>
       </c>
-      <c r="B24" s="2" t="n">
-        <v>0.0049</v>
-      </c>
-      <c r="C24" s="1" t="n">
-        <v>1</v>
-      </c>
-      <c r="D24" s="1" t="s">
+      <c r="E24" s="2" t="n">
+        <v>0.59</v>
+      </c>
+      <c r="F24" s="4" t="s">
         <v>53</v>
-      </c>
-      <c r="E24" s="2" t="n">
-        <v>0.49</v>
       </c>
     </row>
     <row r="25" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -911,7 +918,7 @@
         <v>54</v>
       </c>
       <c r="B25" s="2" t="n">
-        <v>0.005</v>
+        <v>0.0049</v>
       </c>
       <c r="C25" s="1" t="n">
         <v>1</v>
@@ -920,7 +927,7 @@
         <v>55</v>
       </c>
       <c r="E25" s="2" t="n">
-        <v>0.5</v>
+        <v>0.49</v>
       </c>
     </row>
     <row r="26" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -928,7 +935,7 @@
         <v>56</v>
       </c>
       <c r="B26" s="2" t="n">
-        <v>0.0056</v>
+        <v>0.005</v>
       </c>
       <c r="C26" s="1" t="n">
         <v>1</v>
@@ -937,7 +944,7 @@
         <v>57</v>
       </c>
       <c r="E26" s="2" t="n">
-        <v>0.56</v>
+        <v>0.5</v>
       </c>
     </row>
     <row r="27" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -945,7 +952,7 @@
         <v>58</v>
       </c>
       <c r="B27" s="2" t="n">
-        <v>0.0115</v>
+        <v>0.0056</v>
       </c>
       <c r="C27" s="1" t="n">
         <v>1</v>
@@ -954,7 +961,7 @@
         <v>59</v>
       </c>
       <c r="E27" s="2" t="n">
-        <v>0.58</v>
+        <v>0.56</v>
       </c>
     </row>
     <row r="28" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -962,7 +969,7 @@
         <v>60</v>
       </c>
       <c r="B28" s="2" t="n">
-        <v>0.0159</v>
+        <v>0.0115</v>
       </c>
       <c r="C28" s="1" t="n">
         <v>1</v>
@@ -971,7 +978,7 @@
         <v>61</v>
       </c>
       <c r="E28" s="2" t="n">
-        <v>0.8</v>
+        <v>0.58</v>
       </c>
     </row>
     <row r="29" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -979,16 +986,16 @@
         <v>62</v>
       </c>
       <c r="B29" s="2" t="n">
-        <v>0.0087</v>
+        <v>0.0159</v>
       </c>
       <c r="C29" s="1" t="n">
-        <v>4</v>
+        <v>1</v>
       </c>
       <c r="D29" s="1" t="s">
         <v>63</v>
       </c>
       <c r="E29" s="2" t="n">
-        <v>0.44</v>
+        <v>0.8</v>
       </c>
     </row>
     <row r="30" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -996,16 +1003,16 @@
         <v>64</v>
       </c>
       <c r="B30" s="2" t="n">
-        <v>0.4561</v>
+        <v>0.0087</v>
       </c>
       <c r="C30" s="1" t="n">
-        <v>1</v>
+        <v>4</v>
       </c>
       <c r="D30" s="1" t="s">
         <v>65</v>
       </c>
       <c r="E30" s="2" t="n">
-        <v>0.46</v>
+        <v>0.44</v>
       </c>
     </row>
     <row r="31" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -1013,7 +1020,7 @@
         <v>66</v>
       </c>
       <c r="B31" s="2" t="n">
-        <v>6.39</v>
+        <v>0.4561</v>
       </c>
       <c r="C31" s="1" t="n">
         <v>1</v>
@@ -1022,7 +1029,7 @@
         <v>67</v>
       </c>
       <c r="E31" s="2" t="n">
-        <v>6.39</v>
+        <v>0.46</v>
       </c>
     </row>
     <row r="32" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -1030,7 +1037,7 @@
         <v>68</v>
       </c>
       <c r="B32" s="2" t="n">
-        <v>15.99</v>
+        <v>6.39</v>
       </c>
       <c r="C32" s="1" t="n">
         <v>1</v>
@@ -1039,45 +1046,63 @@
         <v>69</v>
       </c>
       <c r="E32" s="2" t="n">
+        <v>6.39</v>
+      </c>
+    </row>
+    <row r="33" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A33" s="1" t="s">
+        <v>70</v>
+      </c>
+      <c r="B33" s="2" t="n">
         <v>15.99</v>
       </c>
-    </row>
-    <row r="33" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="B33" s="2"/>
-      <c r="E33" s="2"/>
+      <c r="C33" s="1" t="n">
+        <v>1</v>
+      </c>
+      <c r="D33" s="1" t="s">
+        <v>71</v>
+      </c>
+      <c r="E33" s="2" t="n">
+        <f aca="false">B33*C33</f>
+        <v>15.99</v>
+      </c>
     </row>
     <row r="34" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A34" s="1" t="s">
-        <v>70</v>
-      </c>
-      <c r="E34" s="2" t="n">
-        <f aca="false">SUM(E2:E32)</f>
-        <v>47.3061</v>
-      </c>
-    </row>
-    <row r="36" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A36" s="1" t="s">
-        <v>71</v>
-      </c>
-      <c r="E36" s="2" t="n">
-        <v>5.3</v>
+      <c r="B34" s="2"/>
+      <c r="E34" s="2"/>
+    </row>
+    <row r="35" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A35" s="1" t="s">
+        <v>72</v>
+      </c>
+      <c r="E35" s="2" t="n">
+        <f aca="false">SUM(E2:E33)</f>
+        <v>47.2772</v>
       </c>
     </row>
     <row r="37" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A37" s="1" t="s">
-        <v>72</v>
+        <v>73</v>
       </c>
       <c r="E37" s="2" t="n">
+        <v>7.3</v>
+      </c>
+    </row>
+    <row r="38" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A38" s="1" t="s">
+        <v>74</v>
+      </c>
+      <c r="E38" s="2" t="n">
         <v>14.56</v>
       </c>
     </row>
-    <row r="39" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A39" s="1" t="s">
-        <v>73</v>
-      </c>
-      <c r="E39" s="2" t="n">
-        <f aca="false">SUM(E34:E37)*1.0825</f>
-        <v>72.70730325</v>
+    <row r="40" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A40" s="1" t="s">
+        <v>75</v>
+      </c>
+      <c r="E40" s="2" t="n">
+        <f aca="false">SUM(E35:E38)*1.0825</f>
+        <v>74.841019</v>
       </c>
     </row>
   </sheetData>

</xml_diff>